<commit_message>
Fase 2: strip OneDrive path metadata from DEPARA.xlsx; drop origin .docx at HEAD
- DEPARA.xlsx carried an <x15ac:absPath> hint pointing at a OneDrive folder
  named after the origin engagement (not visible in any cell). Removed the
  <mc:AlternateContent> block surgically; zip still valid, 0 refs. Original
  kept locally as docs/DEPARA.xlsx.pre-expurgo.bak (gitignored).
- CONTROLE DE ACESSO - FUNÇÕES.xlsx re-scanned: clean, no reference.
- Remove the two origin-branded .docx from HEAD (git filter-repo will also
  drop them from all history in Fase 2b).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DEPARA.xlsx
+++ b/docs/DEPARA.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6629b945a6a46706/Documents/OTB INFORMACOES/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3" documentId="8_{BEC8645C-F7FC-4AA9-986C-7069864B5057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C9A0D25-5C03-4BA3-8A64-EABC89937BAD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76974417-D618-494A-BB2D-9521EF029572}"/>

</xml_diff>